<commit_message>
Changed the email behaviour: instead of all reports having “Chadwicks” in the subject, the reports now use the correct supplier name.
</commit_message>
<xml_diff>
--- a/Airpacks/Airpacks_MATERIAL_PRICES.xlsx
+++ b/Airpacks/Airpacks_MATERIAL_PRICES.xlsx
@@ -28,9 +28,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy hh:mm"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy hh:mm"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -81,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -97,7 +96,8 @@
     </xf>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -646,8 +646,8 @@
           <t>SI-106383</t>
         </is>
       </c>
-      <c r="J2" s="7" t="n">
-        <v>46287.48540836974</v>
+      <c r="J2" s="8" t="n">
+        <v>46287.62051277405</v>
       </c>
     </row>
     <row r="3">
@@ -679,8 +679,8 @@
           <t>SI-106383</t>
         </is>
       </c>
-      <c r="J3" s="7" t="n">
-        <v>46287.48540837016</v>
+      <c r="J3" s="8" t="n">
+        <v>46287.62051277453</v>
       </c>
     </row>
     <row r="4">
@@ -721,8 +721,8 @@
           <t>SI-106121</t>
         </is>
       </c>
-      <c r="J4" s="7" t="n">
-        <v>46287.48540585963</v>
+      <c r="J4" s="8" t="n">
+        <v>46287.62050963873</v>
       </c>
     </row>
     <row r="5">
@@ -763,8 +763,8 @@
           <t>SI-106251</t>
         </is>
       </c>
-      <c r="J5" s="7" t="n">
-        <v>46287.48540701816</v>
+      <c r="J5" s="8" t="n">
+        <v>46287.62051107295</v>
       </c>
     </row>
     <row r="6">
@@ -805,8 +805,8 @@
           <t>SI-106124</t>
         </is>
       </c>
-      <c r="J6" s="7" t="n">
-        <v>46287.48540647698</v>
+      <c r="J6" s="8" t="n">
+        <v>46287.62051042217</v>
       </c>
     </row>
     <row r="7">
@@ -847,8 +847,8 @@
           <t>SI-106121</t>
         </is>
       </c>
-      <c r="J7" s="7" t="n">
-        <v>46287.48540586038</v>
+      <c r="J7" s="8" t="n">
+        <v>46287.62050963972</v>
       </c>
     </row>
     <row r="8">
@@ -880,8 +880,8 @@
           <t>SI-106383</t>
         </is>
       </c>
-      <c r="J8" s="7" t="n">
-        <v>46287.48540837003</v>
+      <c r="J8" s="8" t="n">
+        <v>46287.62051277439</v>
       </c>
     </row>
     <row r="9">
@@ -913,8 +913,8 @@
           <t>SI-105150</t>
         </is>
       </c>
-      <c r="J9" s="7" t="n">
-        <v>46287.48540270795</v>
+      <c r="J9" s="8" t="n">
+        <v>46287.62050527773</v>
       </c>
     </row>
     <row r="10">
@@ -946,8 +946,8 @@
           <t>SI-104976</t>
         </is>
       </c>
-      <c r="J10" s="7" t="n">
-        <v>46287.4854021458</v>
+      <c r="J10" s="8" t="n">
+        <v>46287.62050380234</v>
       </c>
     </row>
     <row r="11">
@@ -979,8 +979,8 @@
           <t>SI-104976</t>
         </is>
       </c>
-      <c r="J11" s="7" t="n">
-        <v>46287.48540214606</v>
+      <c r="J11" s="8" t="n">
+        <v>46287.62050380262</v>
       </c>
     </row>
     <row r="12">
@@ -1012,8 +1012,8 @@
           <t>SI-105459</t>
         </is>
       </c>
-      <c r="J12" s="7" t="n">
-        <v>46287.48540523227</v>
+      <c r="J12" s="8" t="n">
+        <v>46287.62050853067</v>
       </c>
     </row>
     <row r="13">
@@ -1054,8 +1054,8 @@
           <t>SI-106383</t>
         </is>
       </c>
-      <c r="J13" s="7" t="n">
-        <v>46287.48540837028</v>
+      <c r="J13" s="8" t="n">
+        <v>46287.62051277467</v>
       </c>
     </row>
     <row r="14">
@@ -1087,8 +1087,8 @@
           <t>SI-106254</t>
         </is>
       </c>
-      <c r="J14" s="7" t="n">
-        <v>46287.48540766588</v>
+      <c r="J14" s="8" t="n">
+        <v>46287.62051187971</v>
       </c>
     </row>
     <row r="15">
@@ -1129,8 +1129,8 @@
           <t>SI-106254</t>
         </is>
       </c>
-      <c r="J15" s="7" t="n">
-        <v>46287.48540766616</v>
+      <c r="J15" s="8" t="n">
+        <v>46287.62051188001</v>
       </c>
     </row>
     <row r="16">
@@ -1162,8 +1162,8 @@
           <t>SI-105153</t>
         </is>
       </c>
-      <c r="J16" s="7" t="n">
-        <v>46287.48540458349</v>
+      <c r="J16" s="8" t="n">
+        <v>46287.62050756635</v>
       </c>
     </row>
     <row r="17">
@@ -1195,8 +1195,8 @@
           <t>SI-104197</t>
         </is>
       </c>
-      <c r="J17" s="7" t="n">
-        <v>46287.48539914499</v>
+      <c r="J17" s="8" t="n">
+        <v>46287.62049864914</v>
       </c>
     </row>
   </sheetData>
@@ -1412,7 +1412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H277"/>
+  <dimension ref="A1:H291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10269,6 +10269,468 @@
       <c r="G277" t="inlineStr">
         <is>
           <t>SI-106383</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Airpacks</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>C Water Tank Lid 4</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Water Tank Lid 4 48 x 24 x 24 inch CWTJ RIGID LID (5/PK) Cold Water Lagging</t>
+        </is>
+      </c>
+      <c r="E278" t="n">
+        <v>22.29</v>
+      </c>
+      <c r="F278" t="n">
+        <v>15.13</v>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>SI-102779</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Airpacks</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>C Water Tank Lid 1</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Water Tank Lid 1 18 x 12 x 12 inch CWTJ RIGID LID (20/PK) Cold Water</t>
+        </is>
+      </c>
+      <c r="E279" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="F279" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>SI-102779</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Airpacks</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>EWI1200/600/60W200</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>External Wall Insulation White 1200x600x60mm EPS200 Aged</t>
+        </is>
+      </c>
+      <c r="E280" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="F280" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>SI-103298</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Airpacks</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>D&amp;W</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Proofing 4 Q-LON RETRO B BROWN (2.05M) (50/PK) Class 2 (Internal</t>
+        </is>
+      </c>
+      <c r="E281" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="F281" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>SI-103871</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Airpacks</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>D&amp;W</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Proofing 2 Q-LON RETRO 21 B Brown (2.05m) Sealant (50/PK) Class 1</t>
+        </is>
+      </c>
+      <c r="E282" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="F282" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>SI-103871</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>12/06/2026</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Airpacks</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>XPS300/1250/600/60</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>XPS300 - 1250 x 600 x 60mm (7 Sheets per Pack)</t>
+        </is>
+      </c>
+      <c r="E283" t="n">
+        <v>10.86</v>
+      </c>
+      <c r="F283" t="n">
+        <v>10</v>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>SI-104119</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>12/06/2026</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Airpacks</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>EWI1200/600/60W200</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>External Wall Insulation White 1200x600x60mm EPS200 Aged</t>
+        </is>
+      </c>
+      <c r="E284" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="F284" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>SI-104119</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>16/06/2026</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Airpacks</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>D&amp;W</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Proofing 3 Q-LON RETRO B WHITE (2.05M) (50/PK) Class 2 (Internal</t>
+        </is>
+      </c>
+      <c r="E285" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="F285" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>SI-104150</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>16/06/2026</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Airpacks</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>D&amp;W</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Proofing 1 Q-LON RETRO 21 B WHITE (2.05m) Sealant (50/PK) Class 1</t>
+        </is>
+      </c>
+      <c r="E286" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="F286" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>SI-104150</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>16/06/2026</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Airpacks</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>EWI1200/600/60W200</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>External Wall Insulation White 1200x600x60mm EPS200 Aged</t>
+        </is>
+      </c>
+      <c r="E287" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="F287" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>SI-104197</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>17/07/2026</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Airpacks</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>EWI1200/600/60W200</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>External Wall Insulation White 1200x600x60mm EPS200 Aged</t>
+        </is>
+      </c>
+      <c r="E288" t="n">
+        <v>7.13</v>
+      </c>
+      <c r="F288" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>SI-104975</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Airpacks</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>C Water Tank Lid 4</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Water Tank Lid 4 48 x 24 x 24 inch CWTJ RIGID LID (5/PK) Cold Water Lagging</t>
+        </is>
+      </c>
+      <c r="E289" t="n">
+        <v>15.13</v>
+      </c>
+      <c r="F289" t="n">
+        <v>22.29</v>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>SI-106121</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Airpacks</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>C Water Tank Lid 1</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Water Tank Lid 1 18 x 12 x 12 inch CWTJ RIGID LID (20/PK) Cold Water</t>
+        </is>
+      </c>
+      <c r="E290" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="F290" t="n">
+        <v>7.44</v>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>SI-106121</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Airpacks</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>XPS300/1250/600/60</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>XPS300 - 1250 x 600 x 60mm (7 Sheets per Pack)</t>
+        </is>
+      </c>
+      <c r="E291" t="n">
+        <v>10</v>
+      </c>
+      <c r="F291" t="n">
+        <v>10.86</v>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>SI-106124</t>
         </is>
       </c>
     </row>

</xml_diff>